<commit_message>
add vesselexpress and refine others
</commit_message>
<xml_diff>
--- a/Feature_Comparison.xlsx
+++ b/Feature_Comparison.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
   <si>
     <t>Feature</t>
   </si>
@@ -30,6 +30,9 @@
     <t>VesselVio</t>
   </si>
   <si>
+    <t>VesselExpress</t>
+  </si>
+  <si>
     <t>branchpoint_count</t>
   </si>
   <si>
@@ -48,6 +51,30 @@
     <t>no</t>
   </si>
   <si>
+    <t>image_of_branchpoints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">branchpoint image</t>
+  </si>
+  <si>
+    <t>image_of_endpoints</t>
+  </si>
+  <si>
+    <t xml:space="preserve">endpoint image</t>
+  </si>
+  <si>
+    <t>image_of_graph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">graph image</t>
+  </si>
+  <si>
+    <t>max_diffusion_dist_um</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean of the maximum distance from each non-vessel region to the nearest vessel (proxy for oxygen diffusion distance; higher means poorer coverage)</t>
+  </si>
+  <si>
     <t>mean_segment_diam</t>
   </si>
   <si>
@@ -87,7 +114,7 @@
     <t>mean_tortuosity</t>
   </si>
   <si>
-    <t xml:space="preserve">average segment turtosity</t>
+    <t xml:space="preserve">average segment turtosity (segment_length/e2e_distance)</t>
   </si>
   <si>
     <t>mean_tortuosity_bins_0_1_to_20_plus</t>
@@ -102,6 +129,96 @@
     <t xml:space="preserve">branchpoint_count divided by segment_count (network complexity ratio)</t>
   </si>
   <si>
+    <t>per_branchpoint_valency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valency of each branching point (number of incident branches)</t>
+  </si>
+  <si>
+    <t>per_filament_branchpoint_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of branchpoints per filament</t>
+  </si>
+  <si>
+    <t>per_filament_endpoint_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of endpoints per filament</t>
+  </si>
+  <si>
+    <t>per_filament_segment_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of segments per filament</t>
+  </si>
+  <si>
+    <t>per_segment_branching_angle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">angle betw. segment and its predecessor at the branching point for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_branching_points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of branching points incident to each segment (0–2)</t>
+  </si>
+  <si>
+    <t>per_segment_diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mean vessel diameter measured along centerlines for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_mean_radius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">average radius along the segment centerline for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_min_radius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">minimum radius along the segment for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_radius_stddev</t>
+  </si>
+  <si>
+    <t xml:space="preserve">standard deviation of radii along the segment for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_straightness</t>
+  </si>
+  <si>
+    <t xml:space="preserve">straightness (e2e_distance/segment_length) for each vessel segment</t>
+  </si>
+  <si>
+    <t>per_segment_terminal_points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of terminal points incident to each segment (0-2)</t>
+  </si>
+  <si>
+    <t>per_segment_vessel_length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">centerline length for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">volume of each vessel segment</t>
+  </si>
+  <si>
+    <t>per_sgement_max_radius</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximum radius along the segment for each segment</t>
+  </si>
+  <si>
     <t>roi_volume</t>
   </si>
   <si>
@@ -126,6 +243,12 @@
     <t xml:space="preserve">distribution of segment sizes across radius bins</t>
   </si>
   <si>
+    <t>skeleton_as_graphml</t>
+  </si>
+  <si>
+    <t xml:space="preserve">export of the skeleton graph</t>
+  </si>
+  <si>
     <t>skeleton_surface_area</t>
   </si>
   <si>
@@ -138,7 +261,7 @@
     <t xml:space="preserve">fraction of image pixels classified as vessel</t>
   </si>
   <si>
-    <t xml:space="preserve">yes (volume)</t>
+    <t xml:space="preserve">yes (Total network volume (3D) or total PAF (2D) is reported as “Volume” / “Percent Area Fraction (PAF) %)</t>
   </si>
   <si>
     <t>vessel_length</t>
@@ -195,11 +318,14 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -661,8 +787,9 @@
   <sheetFormatPr baseColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="39.7109375"/>
-    <col customWidth="1" min="2" max="2" width="68.28125"/>
-    <col customWidth="1" min="4" max="4" width="19.7109375"/>
+    <col customWidth="1" min="2" max="2" width="70.7109375"/>
+    <col customWidth="1" min="4" max="4" width="12.421875"/>
+    <col customWidth="1" min="5" max="5" width="13.28125"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -678,280 +805,723 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>6</v>
+        <v>14</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" t="s">
-        <v>6</v>
+        <v>16</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" t="s">
         <v>17</v>
       </c>
+      <c r="B7" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="E7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D10" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C12" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="3" t="s">
         <v>31</v>
       </c>
+      <c r="B14" t="s">
+        <v>32</v>
+      </c>
       <c r="C14" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D14" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>6</v>
+        <v>7</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" t="s">
-        <v>36</v>
-      </c>
-      <c r="B17" t="s">
         <v>37</v>
       </c>
-      <c r="C17" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" t="s">
-        <v>6</v>
+      <c r="B17" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" t="s">
-        <v>38</v>
+      <c r="A18" s="3" t="s">
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C18" t="s">
-        <v>6</v>
+        <v>40</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="D18" t="s">
-        <v>40</v>
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="19" ht="14.25">
-      <c r="A19" t="s">
+      <c r="A19" s="3" t="s">
         <v>41</v>
       </c>
       <c r="B19" t="s">
         <v>42</v>
       </c>
-      <c r="C19" t="s">
-        <v>6</v>
+      <c r="C19" s="3" t="s">
+        <v>10</v>
       </c>
       <c r="D19" t="s">
+        <v>10</v>
+      </c>
+      <c r="E19" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="A20" s="3" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="20" ht="14.25">
-      <c r="A20" t="s">
+      <c r="B20" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" t="s">
+        <v>10</v>
+      </c>
+      <c r="E20" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="A21" t="s">
         <v>45</v>
       </c>
-      <c r="C20" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" t="s">
-        <v>9</v>
-      </c>
+      <c r="B21" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E21" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="A22" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" t="s">
+        <v>48</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E22" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="A23" t="s">
+        <v>49</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
+        <v>10</v>
+      </c>
+      <c r="D23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C24" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" ht="14.25">
+      <c r="A25" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" ht="14.25">
+      <c r="A26" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="A27" t="s">
+        <v>57</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" ht="14.25">
+      <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E28" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" ht="14.25">
+      <c r="A29" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" t="s">
+        <v>10</v>
+      </c>
+      <c r="D29" t="s">
+        <v>7</v>
+      </c>
+      <c r="E29" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" ht="14.25">
+      <c r="A30" t="s">
+        <v>63</v>
+      </c>
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+      <c r="C30" t="s">
+        <v>10</v>
+      </c>
+      <c r="D30" t="s">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" ht="14.25">
+      <c r="A31" t="s">
+        <v>65</v>
+      </c>
+      <c r="B31" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E31" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32" ht="14.25">
+      <c r="A32" t="s">
+        <v>67</v>
+      </c>
+      <c r="B32" t="s">
+        <v>68</v>
+      </c>
+      <c r="C32" t="s">
+        <v>10</v>
+      </c>
+      <c r="D32" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" ht="14.25">
+      <c r="A33" t="s">
+        <v>69</v>
+      </c>
+      <c r="B33" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" t="s">
+        <v>7</v>
+      </c>
+      <c r="D33" t="s">
+        <v>7</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" ht="14.25">
+      <c r="A34" t="s">
+        <v>71</v>
+      </c>
+      <c r="B34" t="s">
+        <v>72</v>
+      </c>
+      <c r="C34" t="s">
+        <v>10</v>
+      </c>
+      <c r="D34" t="s">
+        <v>7</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" ht="14.25">
+      <c r="A35" t="s">
+        <v>73</v>
+      </c>
+      <c r="B35" t="s">
+        <v>74</v>
+      </c>
+      <c r="C35" t="s">
+        <v>10</v>
+      </c>
+      <c r="D35" t="s">
+        <v>7</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" ht="14.25">
+      <c r="A36" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" t="s">
+        <v>7</v>
+      </c>
+      <c r="E36" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" ht="14.25">
+      <c r="A37" t="s">
+        <v>77</v>
+      </c>
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" t="s">
+        <v>10</v>
+      </c>
+      <c r="D37" t="s">
+        <v>7</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="A38" t="s">
+        <v>79</v>
+      </c>
+      <c r="B38" t="s">
+        <v>80</v>
+      </c>
+      <c r="C38" t="s">
+        <v>7</v>
+      </c>
+      <c r="D38" t="s">
+        <v>81</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" ht="14.25">
+      <c r="A39" t="s">
+        <v>82</v>
+      </c>
+      <c r="B39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C39" t="s">
+        <v>7</v>
+      </c>
+      <c r="D39" t="s">
+        <v>84</v>
+      </c>
+      <c r="E39" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" ht="14.25">
+      <c r="A40" t="s">
+        <v>85</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C40" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="A41" s="3"/>
     </row>
   </sheetData>
-  <sortState ref="A2:D20" columnSort="0">
-    <sortCondition sortBy="value" descending="0" ref="A2:A20"/>
+  <sortState ref="A2:E40" columnSort="0">
+    <sortCondition sortBy="value" descending="0" ref="A2:A40"/>
   </sortState>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{007400CB-002F-4EEE-9ECB-00F600A30097}">
+            <xm:f>LEFT(C1,LEN("yes"))="yes"</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF006100"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>C1:F32 F33:F35 C36:F36 E37:F39 C40:F40 C33:D33 C34:D34 C35:D35 E33 E34 E35 D37 D38 D39 C37 C38 C39</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="containsText" priority="1" text="no" id="{00FC0040-00B0-4929-BC67-00F300C4006D}">
+            <xm:f>NOT(ISERROR(SEARCH("no",C1)))</xm:f>
+            <x14:dxf>
+              <font>
+                <color rgb="FF9C0006"/>
+              </font>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>C1:F32 F33:F35 C36:F36 E37:F39 C40:F48 C33:D33 C34:D34 C35:D35 E33 E34 E35 D37 D38 D39 C37 C38 C39</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add current vesskel features
</commit_message>
<xml_diff>
--- a/Feature_Comparison.xlsx
+++ b/Feature_Comparison.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
   <si>
     <t>Feature</t>
   </si>
@@ -39,6 +39,9 @@
     <t>VesSAP</t>
   </si>
   <si>
+    <t>VesSkel</t>
+  </si>
+  <si>
     <t>alignment_coherency_percent</t>
   </si>
   <si>
@@ -57,6 +60,12 @@
     <t xml:space="preserve">number of branching points in the skeleton</t>
   </si>
   <si>
+    <t>component_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of connected components in the skeleton graph</t>
+  </si>
+  <si>
     <t>endpoint_count</t>
   </si>
   <si>
@@ -69,6 +78,12 @@
     <t xml:space="preserve">box counting fractal dimension of the skeletonized mask</t>
   </si>
   <si>
+    <t>fractal_dimension_r2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">box counting fractal dimension r^2 of the skeletonized mask</t>
+  </si>
+  <si>
     <t>gap_area_p5</t>
   </si>
   <si>
@@ -132,6 +147,18 @@
     <t xml:space="preserve">mean of the maximum distance from each non-vessel region to the nearest vessel (proxy for oxygen diffusion distance; higher means poorer coverage)</t>
   </si>
   <si>
+    <t>max_segment_length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximum centerline path length among all segments</t>
+  </si>
+  <si>
+    <t>max_valency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximum node degree</t>
+  </si>
+  <si>
     <t>mean_curvature</t>
   </si>
   <si>
@@ -198,6 +225,18 @@
     <t xml:space="preserve">branchpoint_count divided by segment_count (network complexity ratio)</t>
   </si>
   <si>
+    <t>min_segment_length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">minimum centerline path length among all segments</t>
+  </si>
+  <si>
+    <t>node_count</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number of unique nodes (vertices) in the skeleton graph</t>
+  </si>
+  <si>
     <t>per_branchpoint_valency</t>
   </si>
   <si>
@@ -228,6 +267,12 @@
     <t xml:space="preserve">per-gap array: individual inscribed gap circle areas, one row per detected gap (px)</t>
   </si>
   <si>
+    <t>per_segment_branch_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0=junction-junction, 1=junction-endpoint, 2=endpoint-endpoint</t>
+  </si>
+  <si>
     <t>per_segment_branching_angle</t>
   </si>
   <si>
@@ -246,6 +291,12 @@
     <t xml:space="preserve">mean vessel diameter measured along centerlines for each segment</t>
   </si>
   <si>
+    <t>per_segment_euclidean_distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">straight-line end-to-end distance for each segment</t>
+  </si>
+  <si>
     <t>per_segment_mean_radius</t>
   </si>
   <si>
@@ -276,12 +327,21 @@
     <t xml:space="preserve">number of terminal points incident to each segment (0-2)</t>
   </si>
   <si>
+    <t>per_segment_tortuosity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tortuosity for each segment (branch-distance / euclidean-distance)</t>
+  </si>
+  <si>
     <t>per_segment_vessel_length</t>
   </si>
   <si>
     <t xml:space="preserve">centerline length for each segment</t>
   </si>
   <si>
+    <t xml:space="preserve">centerline path length along the skeleton for each segment</t>
+  </si>
+  <si>
     <t>per_segment_volume</t>
   </si>
   <si>
@@ -340,6 +400,18 @@
   </si>
   <si>
     <t xml:space="preserve">standard deviation of inscribed gap circle areas (px)</t>
+  </si>
+  <si>
+    <t>stddev_segment_length</t>
+  </si>
+  <si>
+    <t xml:space="preserve">standard deviation of segment centerline lengths</t>
+  </si>
+  <si>
+    <t>stddev_tortuosity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">standard deviation of per-segment tortuosity</t>
   </si>
   <si>
     <t>vessel_area</t>
@@ -908,258 +980,294 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H4" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" s="4" t="s">
+      <c r="A5" t="s">
         <v>16</v>
       </c>
+      <c r="B5" t="s">
+        <v>17</v>
+      </c>
       <c r="C5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="s">
+      <c r="A6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
+      <c r="B6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>10</v>
+        <v>10</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H6" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" t="s">
-        <v>19</v>
+      <c r="A7" s="4" t="s">
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>9</v>
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>10</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" s="4" t="s">
         <v>24</v>
       </c>
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
       <c r="C9" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G9" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="4" t="s">
-        <v>25</v>
+      <c r="A10" t="s">
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>10</v>
+        <v>10</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" t="s">
         <v>28</v>
       </c>
+      <c r="B11" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="C11" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F11" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" t="s">
-        <v>29</v>
+      <c r="F11" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" t="s">
+      <c r="A12" s="4" t="s">
         <v>30</v>
       </c>
       <c r="B12" t="s">
         <v>31</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E12" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="13" ht="14.25">
@@ -1170,979 +1278,1405 @@
         <v>33</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>29</v>
+        <v>34</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="14" ht="14.25">
-      <c r="A14" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B14" s="4" t="s">
+      <c r="A14" t="s">
         <v>35</v>
       </c>
-      <c r="C14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D14" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" t="s">
-        <v>9</v>
+      <c r="B14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>29</v>
+        <v>10</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" t="s">
-        <v>36</v>
-      </c>
-      <c r="B15" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="C15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" t="s">
-        <v>9</v>
+      <c r="B15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>9</v>
+        <v>34</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" t="s">
-        <v>38</v>
+      <c r="A16" s="4" t="s">
+        <v>39</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>9</v>
+        <v>40</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" t="s">
+        <v>10</v>
       </c>
       <c r="F16" t="s">
         <v>10</v>
       </c>
-      <c r="G16" s="4" t="s">
-        <v>9</v>
+      <c r="G16" t="s">
+        <v>34</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="17" ht="14.25">
       <c r="A17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>9</v>
+      <c r="B17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="18" ht="14.25">
       <c r="A18" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" t="s">
         <v>43</v>
       </c>
-      <c r="C18" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" t="s">
-        <v>9</v>
+      <c r="B18" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F18" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="19" ht="14.25">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H19" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="20" ht="14.25">
       <c r="A20" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" t="s">
         <v>47</v>
       </c>
-      <c r="C20" t="s">
-        <v>9</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="B20" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H20" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="21" ht="14.25">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" t="s">
-        <v>9</v>
-      </c>
-      <c r="D21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="F21" s="4" t="s">
+        <v>11</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H21" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="22" ht="14.25">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G22" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H22" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="23" ht="14.25">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C23" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D23" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G23" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H23" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="24" ht="14.25">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C24" t="s">
         <v>10</v>
       </c>
       <c r="D24" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="25" ht="14.25">
       <c r="A25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B25" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D25" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G25" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="26" ht="14.25">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C26" t="s">
         <v>10</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H26" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="27" ht="14.25">
       <c r="A27" t="s">
-        <v>60</v>
-      </c>
-      <c r="B27" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E27" t="s">
+      <c r="B27" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" t="s">
+        <v>11</v>
+      </c>
+      <c r="E27" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="4" t="s">
-        <v>62</v>
+      <c r="A28" t="s">
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>9</v>
+        <v>64</v>
+      </c>
+      <c r="C28" t="s">
+        <v>11</v>
       </c>
       <c r="D28" t="s">
-        <v>9</v>
-      </c>
-      <c r="E28" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="4" t="s">
-        <v>64</v>
+      <c r="A29" t="s">
+        <v>65</v>
       </c>
       <c r="B29" t="s">
-        <v>65</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>9</v>
+        <v>66</v>
+      </c>
+      <c r="C29" t="s">
+        <v>10</v>
       </c>
       <c r="D29" t="s">
-        <v>9</v>
-      </c>
-      <c r="E29" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H29" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="4" t="s">
-        <v>66</v>
+      <c r="A30" t="s">
+        <v>67</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>9</v>
+        <v>68</v>
+      </c>
+      <c r="C30" t="s">
+        <v>11</v>
       </c>
       <c r="D30" t="s">
-        <v>9</v>
-      </c>
-      <c r="E30" t="s">
+        <v>10</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H30" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="31" ht="14.25">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="32" ht="14.25">
       <c r="A32" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E32" t="s">
-        <v>10</v>
-      </c>
-      <c r="F32" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H32" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="33" ht="14.25">
       <c r="A33" t="s">
-        <v>72</v>
-      </c>
-      <c r="B33" t="s">
         <v>73</v>
       </c>
+      <c r="B33" s="4" t="s">
+        <v>74</v>
+      </c>
       <c r="C33" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E33" t="s">
-        <v>10</v>
-      </c>
-      <c r="F33" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F33" t="s">
+        <v>10</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H33" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" t="s">
-        <v>74</v>
-      </c>
-      <c r="B34" s="4" t="s">
+      <c r="A34" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C34" t="s">
-        <v>9</v>
+      <c r="B34" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E34" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
       </c>
       <c r="G34" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" t="s">
-        <v>76</v>
-      </c>
-      <c r="B35" s="4" t="s">
+      <c r="A35" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C35" t="s">
-        <v>9</v>
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
       </c>
       <c r="E35" t="s">
-        <v>9</v>
-      </c>
-      <c r="F35" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F35" t="s">
+        <v>10</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" t="s">
-        <v>78</v>
-      </c>
-      <c r="B36" s="4" t="s">
+      <c r="A36" s="4" t="s">
         <v>79</v>
       </c>
+      <c r="B36" t="s">
+        <v>80</v>
+      </c>
       <c r="C36" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D36" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D36" t="s">
         <v>10</v>
       </c>
       <c r="E36" t="s">
-        <v>9</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F36" t="s">
+        <v>10</v>
       </c>
       <c r="G36" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="37" ht="14.25">
       <c r="A37" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E37" t="s">
-        <v>9</v>
+      <c r="E37" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G37" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="38" ht="14.25">
       <c r="A38" t="s">
-        <v>82</v>
-      </c>
-      <c r="B38" s="4" t="s">
         <v>83</v>
       </c>
+      <c r="B38" t="s">
+        <v>84</v>
+      </c>
       <c r="C38" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H38" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="39" ht="14.25">
       <c r="A39" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E39" t="s">
-        <v>10</v>
-      </c>
-      <c r="F39" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="F39" t="s">
+        <v>10</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H39" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="40" ht="14.25">
       <c r="A40" t="s">
-        <v>86</v>
-      </c>
-      <c r="B40" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="C40" t="s">
-        <v>9</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="B40" t="s">
+        <v>88</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D40" s="4" t="s">
         <v>10</v>
       </c>
       <c r="E40" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H40" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="41" ht="14.25">
       <c r="A41" t="s">
-        <v>88</v>
-      </c>
-      <c r="B41" t="s">
         <v>89</v>
       </c>
+      <c r="B41" s="4" t="s">
+        <v>90</v>
+      </c>
       <c r="C41" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D41" t="s">
         <v>10</v>
       </c>
       <c r="E41" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="42" ht="14.25">
       <c r="A42" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D42" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E42" t="s">
-        <v>9</v>
+      <c r="E42" s="4" t="s">
+        <v>10</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H42" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="43" ht="14.25">
       <c r="A43" t="s">
-        <v>92</v>
-      </c>
-      <c r="B43" t="s">
         <v>93</v>
       </c>
+      <c r="B43" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="C43" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D43" t="s">
-        <v>10</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="44" ht="14.25">
       <c r="A44" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C44" t="s">
-        <v>10</v>
-      </c>
-      <c r="D44" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D44" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" t="s">
         <v>10</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="45" ht="14.25">
       <c r="A45" t="s">
-        <v>96</v>
-      </c>
-      <c r="B45" t="s">
         <v>97</v>
       </c>
-      <c r="C45" t="s">
-        <v>9</v>
-      </c>
-      <c r="D45" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" s="4" t="s">
-        <v>9</v>
+      <c r="B45" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" t="s">
+        <v>10</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B46" t="s">
+      <c r="A46" t="s">
         <v>99</v>
       </c>
+      <c r="B46" s="4" t="s">
+        <v>100</v>
+      </c>
       <c r="C46" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E46" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F46" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="47" ht="14.25">
       <c r="A47" t="s">
-        <v>100</v>
-      </c>
-      <c r="B47" t="s">
         <v>101</v>
       </c>
-      <c r="C47" t="s">
-        <v>9</v>
-      </c>
-      <c r="D47" t="s">
-        <v>10</v>
-      </c>
-      <c r="E47" s="4" t="s">
-        <v>9</v>
+      <c r="B47" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E47" t="s">
+        <v>11</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G47" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="48" ht="14.25">
       <c r="A48" t="s">
-        <v>102</v>
-      </c>
-      <c r="B48" t="s">
         <v>103</v>
       </c>
-      <c r="C48" t="s">
-        <v>9</v>
-      </c>
-      <c r="D48" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" t="s">
+      <c r="B48" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="4" t="s">
         <v>10</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H48" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="49" ht="14.25">
       <c r="A49" t="s">
-        <v>104</v>
-      </c>
-      <c r="B49" t="s">
         <v>105</v>
       </c>
+      <c r="B49" s="4" t="s">
+        <v>106</v>
+      </c>
       <c r="C49" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D49" t="s">
-        <v>10</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="E49" t="s">
+        <v>11</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H49" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="50" ht="14.25">
       <c r="A50" t="s">
-        <v>106</v>
-      </c>
-      <c r="B50" t="s">
+        <v>105</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>107</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F50" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="51" ht="14.25">
       <c r="A51" t="s">
         <v>108</v>
       </c>
-      <c r="B51" s="4" t="s">
+      <c r="B51" t="s">
         <v>109</v>
       </c>
-      <c r="C51" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D51" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F51" t="s">
+      <c r="C51" t="s">
+        <v>10</v>
+      </c>
+      <c r="D51" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H51" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="52" ht="14.25">
       <c r="A52" t="s">
         <v>110</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="C52" t="s">
-        <v>10</v>
-      </c>
-      <c r="D52" t="s">
-        <v>112</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>9</v>
+      <c r="C52" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" t="s">
+        <v>10</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="53" ht="14.25">
       <c r="A53" t="s">
+        <v>112</v>
+      </c>
+      <c r="B53" t="s">
         <v>113</v>
       </c>
-      <c r="B53" t="s">
-        <v>114</v>
-      </c>
       <c r="C53" t="s">
         <v>10</v>
       </c>
       <c r="D53" t="s">
-        <v>115</v>
-      </c>
-      <c r="E53" t="s">
-        <v>9</v>
-      </c>
-      <c r="F53" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" s="4" t="s">
         <v>10</v>
       </c>
       <c r="G53" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="54" ht="14.25">
       <c r="A54" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="C54" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="55" ht="14.25">
+      <c r="A55" t="s">
         <v>116</v>
       </c>
-      <c r="B54" s="4" t="s">
+      <c r="B55" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="C54" t="s">
-        <v>10</v>
-      </c>
-      <c r="D54" t="s">
-        <v>9</v>
-      </c>
-      <c r="E54" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F54" t="s">
-        <v>9</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="55" ht="14.25">
-      <c r="A55"/>
+      <c r="C55" t="s">
+        <v>10</v>
+      </c>
+      <c r="D55" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="56" ht="14.25">
-      <c r="A56"/>
+      <c r="A56" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B56" t="s">
+        <v>119</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>11</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="57" ht="14.25">
-      <c r="A57"/>
+      <c r="A57" t="s">
+        <v>120</v>
+      </c>
+      <c r="B57" t="s">
+        <v>121</v>
+      </c>
+      <c r="C57" t="s">
+        <v>10</v>
+      </c>
+      <c r="D57" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="58" ht="14.25">
-      <c r="A58"/>
+      <c r="A58" t="s">
+        <v>122</v>
+      </c>
+      <c r="B58" t="s">
+        <v>123</v>
+      </c>
+      <c r="C58" t="s">
+        <v>10</v>
+      </c>
+      <c r="D58" t="s">
+        <v>11</v>
+      </c>
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="59" ht="14.25">
+      <c r="A59" t="s">
+        <v>124</v>
+      </c>
+      <c r="B59" t="s">
+        <v>125</v>
+      </c>
+      <c r="C59" t="s">
+        <v>10</v>
+      </c>
+      <c r="D59" t="s">
+        <v>11</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="60" ht="14.25">
+      <c r="A60" t="s">
+        <v>126</v>
+      </c>
+      <c r="B60" t="s">
+        <v>127</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="61" ht="14.25">
+      <c r="A61" t="s">
+        <v>128</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62" ht="14.25">
+      <c r="A62" t="s">
+        <v>130</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H62" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="63" ht="14.25">
+      <c r="A63" t="s">
+        <v>132</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E63" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F63" t="s">
+        <v>11</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="64" ht="14.25">
+      <c r="A64" t="s">
+        <v>134</v>
+      </c>
+      <c r="B64" t="s">
+        <v>135</v>
+      </c>
+      <c r="C64" t="s">
+        <v>11</v>
+      </c>
+      <c r="D64" t="s">
+        <v>136</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H64" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65" ht="14.25">
+      <c r="A65" t="s">
+        <v>137</v>
+      </c>
+      <c r="B65" t="s">
+        <v>138</v>
+      </c>
+      <c r="C65" t="s">
+        <v>11</v>
+      </c>
+      <c r="D65" t="s">
+        <v>139</v>
+      </c>
+      <c r="E65" t="s">
+        <v>10</v>
+      </c>
+      <c r="F65" t="s">
+        <v>11</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="66" ht="14.25">
+      <c r="A66" t="s">
+        <v>140</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="C66" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" t="s">
+        <v>10</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
-  <sortState ref="A2:G54" columnSort="0">
-    <sortCondition sortBy="value" descending="0" ref="A2:A54"/>
+  <sortState ref="A2:H66" columnSort="0">
+    <sortCondition sortBy="value" descending="0" ref="A2:A66"/>
   </sortState>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -2152,7 +2686,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{00B500BB-0079-4CF5-A615-0091002700FE}">
+          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{00D6004E-00B0-4242-AD7D-0020002000C6}">
             <xm:f>LEFT(C1,LEN("yes"))="yes"</xm:f>
             <x14:dxf>
               <font>
@@ -2166,11 +2700,11 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>C2:G54</xm:sqref>
+          <xm:sqref>C2:H66</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" text="no" id="{00660067-0096-4664-9DD3-006100820007}">
-            <xm:f>NOT(ISERROR(SEARCH("no",C1)))</xm:f>
+          <x14:cfRule type="beginsWith" priority="1" text="no" id="{0016008F-002E-423C-8287-005D002F0030}">
+            <xm:f>LEFT(C2,LEN("no"))="no"</xm:f>
             <x14:dxf>
               <font>
                 <color rgb="FF9C0006"/>
@@ -2183,7 +2717,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>C2:G54</xm:sqref>
+          <xm:sqref>C2:H66</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
add some general features
</commit_message>
<xml_diff>
--- a/Feature_Comparison.xlsx
+++ b/Feature_Comparison.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204">
   <si>
     <t>Feature</t>
   </si>
@@ -511,6 +511,123 @@
   </si>
   <si>
     <t xml:space="preserve">centerline length per image area</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>2D/3D</t>
+  </si>
+  <si>
+    <t>2D</t>
+  </si>
+  <si>
+    <t>both</t>
+  </si>
+  <si>
+    <t>3D</t>
+  </si>
+  <si>
+    <t>License</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSD  3.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GPLv. 3</t>
+  </si>
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>MIT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSD 3-clause</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input Type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw 2D fluorescent images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-binarized datasets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw 3D Volumes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw 2D Images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw 3D Volume</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-segmented binary mask</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pre-skeletonized binary</t>
+  </si>
+  <si>
+    <t>Segmentation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto (background sub + adaptive threshold + morphological)</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto (dual Frangi filter + statistical threshold)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto (Steger ridge detection)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto (5-layer 3D CNN, transfer learning)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None (requires pre-segmented input)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None (skeleton analysis only)</t>
+  </si>
+  <si>
+    <t>Skeletonization</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matlab bwmorph</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lee94 (custom numba impl)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">skimage lee94</t>
+  </si>
+  <si>
+    <t>GUI/Interface</t>
+  </si>
+  <si>
+    <t xml:space="preserve">interactive Matlab GUI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PyQt5 standalone app + cli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Web App (Docker) and Napari Plugin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FIJI/ImageJ Plugin with guided param setup</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLI only</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLI + napari Plugin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Napari Plugin and Python Package</t>
   </si>
 </sst>
 </file>
@@ -552,11 +669,9 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1021,8 +1136,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="39.7109375"/>
-    <col customWidth="1" min="2" max="2" width="70.7109375"/>
+    <col customWidth="1" min="1" max="1" width="27.7109375"/>
+    <col customWidth="1" min="2" max="2" width="51.421875"/>
     <col customWidth="1" min="4" max="4" width="12.421875"/>
     <col customWidth="1" min="5" max="5" width="13.28125"/>
   </cols>
@@ -1484,7 +1599,7 @@
       <c r="G16" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="H16" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I16" s="2" t="s">
@@ -1492,7 +1607,7 @@
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B17" t="s">
@@ -1524,7 +1639,7 @@
       <c r="A18" t="s">
         <v>44</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="3" t="s">
         <v>45</v>
       </c>
       <c r="C18" t="s">
@@ -1542,10 +1657,10 @@
       <c r="G18" t="s">
         <v>11</v>
       </c>
-      <c r="H18" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I18" s="3" t="s">
+      <c r="H18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1553,7 +1668,7 @@
       <c r="A19" t="s">
         <v>46</v>
       </c>
-      <c r="B19" s="4" t="s">
+      <c r="B19" s="2" t="s">
         <v>47</v>
       </c>
       <c r="C19" t="s">
@@ -1594,7 +1709,7 @@
       <c r="E20" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="4" t="s">
+      <c r="F20" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G20" t="s">
@@ -1603,7 +1718,7 @@
       <c r="H20" t="s">
         <v>12</v>
       </c>
-      <c r="I20" s="4" t="s">
+      <c r="I20" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1611,7 +1726,7 @@
       <c r="A21" t="s">
         <v>50</v>
       </c>
-      <c r="B21" s="4" t="s">
+      <c r="B21" s="2" t="s">
         <v>51</v>
       </c>
       <c r="C21" t="s">
@@ -1632,7 +1747,7 @@
       <c r="H21" t="s">
         <v>11</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1643,16 +1758,16 @@
       <c r="B22" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="4" t="s">
+      <c r="C22" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E22" t="s">
         <v>11</v>
       </c>
-      <c r="F22" s="4" t="s">
+      <c r="F22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="G22" t="s">
@@ -1661,7 +1776,7 @@
       <c r="H22" t="s">
         <v>11</v>
       </c>
-      <c r="I22" s="4" t="s">
+      <c r="I22" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1687,10 +1802,10 @@
       <c r="G23" t="s">
         <v>11</v>
       </c>
-      <c r="H23" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I23" s="3" t="s">
+      <c r="H23" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I23" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1719,7 +1834,7 @@
       <c r="H24" t="s">
         <v>12</v>
       </c>
-      <c r="I24" s="4" t="s">
+      <c r="I24" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1832,10 +1947,10 @@
       <c r="G28" t="s">
         <v>11</v>
       </c>
-      <c r="H28" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" s="3" t="s">
+      <c r="H28" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1864,7 +1979,7 @@
       <c r="H29" t="s">
         <v>12</v>
       </c>
-      <c r="I29" s="4" t="s">
+      <c r="I29" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1893,7 +2008,7 @@
       <c r="H30" t="s">
         <v>11</v>
       </c>
-      <c r="I30" s="3" t="s">
+      <c r="I30" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1968,10 +2083,10 @@
       <c r="D33" t="s">
         <v>11</v>
       </c>
-      <c r="E33" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F33" s="4" t="s">
+      <c r="E33" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G33" t="s">
@@ -1988,13 +2103,13 @@
       <c r="A34" t="s">
         <v>76</v>
       </c>
-      <c r="B34" s="4" t="s">
+      <c r="B34" s="2" t="s">
         <v>77</v>
       </c>
       <c r="C34" t="s">
         <v>11</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D34" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E34" t="s">
@@ -2009,7 +2124,7 @@
       <c r="H34" t="s">
         <v>11</v>
       </c>
-      <c r="I34" s="4" t="s">
+      <c r="I34" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2072,7 +2187,7 @@
       </c>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="4" t="s">
+      <c r="A37" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B37" t="s">
@@ -2104,7 +2219,7 @@
       <c r="A38" t="s">
         <v>84</v>
       </c>
-      <c r="B38" s="4" t="s">
+      <c r="B38" s="2" t="s">
         <v>85</v>
       </c>
       <c r="C38" t="s">
@@ -2122,24 +2237,24 @@
       <c r="G38" t="s">
         <v>11</v>
       </c>
-      <c r="H38" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I38" s="3" t="s">
+      <c r="H38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I38" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="4" t="s">
+      <c r="A39" s="2" t="s">
         <v>86</v>
       </c>
       <c r="B39" t="s">
         <v>87</v>
       </c>
-      <c r="C39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D39" s="3" t="s">
+      <c r="C39" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E39" s="2" t="s">
@@ -2148,10 +2263,10 @@
       <c r="F39" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H39" s="3" t="s">
+      <c r="G39" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H39" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I39" s="2" t="s">
@@ -2159,31 +2274,31 @@
       </c>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="4" t="s">
+      <c r="A40" s="2" t="s">
         <v>88</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D40" s="3" t="s">
+      <c r="C40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H40" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I40" s="3" t="s">
+      <c r="F40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I40" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2194,13 +2309,13 @@
       <c r="B41" t="s">
         <v>91</v>
       </c>
-      <c r="C41" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E41" s="4" t="s">
+      <c r="C41" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F41" t="s">
@@ -2212,7 +2327,7 @@
       <c r="H41" t="s">
         <v>12</v>
       </c>
-      <c r="I41" s="4" t="s">
+      <c r="I41" s="2" t="s">
         <v>92</v>
       </c>
     </row>
@@ -2238,10 +2353,10 @@
       <c r="G42" t="s">
         <v>11</v>
       </c>
-      <c r="H42" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I42" s="3" t="s">
+      <c r="H42" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I42" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2252,10 +2367,10 @@
       <c r="B43" t="s">
         <v>96</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D43" s="4" t="s">
+      <c r="C43" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D43" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E43" t="s">
@@ -2270,33 +2385,33 @@
       <c r="H43" t="s">
         <v>11</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="I43" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="44" ht="14.25">
-      <c r="A44" s="4" t="s">
+      <c r="A44" s="2" t="s">
         <v>97</v>
       </c>
       <c r="B44" t="s">
         <v>98</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D44" s="3" t="s">
+      <c r="C44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H44" s="3" t="s">
+      <c r="F44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H44" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I44" s="2" t="s">
@@ -2333,31 +2448,31 @@
       </c>
     </row>
     <row r="46" ht="14.25">
-      <c r="A46" s="4" t="s">
+      <c r="A46" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B46" s="3" t="s">
+      <c r="B46" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C46" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D46" s="3" t="s">
+      <c r="C46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F46" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I46" s="3" t="s">
+      <c r="F46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I46" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2374,7 +2489,7 @@
       <c r="D47" t="s">
         <v>11</v>
       </c>
-      <c r="E47" s="4" t="s">
+      <c r="E47" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F47" t="s">
@@ -2391,42 +2506,42 @@
       </c>
     </row>
     <row r="48" ht="14.25">
-      <c r="A48" s="4" t="s">
+      <c r="A48" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B48" s="3" t="s">
+      <c r="B48" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F48" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="3" t="s">
+      <c r="C48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G48" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H48" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="I48" s="3" t="s">
+      <c r="I48" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="49" ht="14.25">
-      <c r="A49" s="4" t="s">
+      <c r="A49" s="2" t="s">
         <v>107</v>
       </c>
       <c r="B49" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D49" s="2" t="s">
@@ -2435,10 +2550,10 @@
       <c r="E49" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="F49" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G49" s="3" t="s">
+      <c r="F49" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G49" s="2" t="s">
         <v>11</v>
       </c>
       <c r="H49" s="2" t="s">
@@ -2452,7 +2567,7 @@
       <c r="A50" t="s">
         <v>109</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="B50" s="2" t="s">
         <v>110</v>
       </c>
       <c r="C50" t="s">
@@ -2470,7 +2585,7 @@
       <c r="G50" t="s">
         <v>11</v>
       </c>
-      <c r="H50" s="4" t="s">
+      <c r="H50" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="s">
@@ -2507,10 +2622,10 @@
       </c>
     </row>
     <row r="52" ht="14.25">
-      <c r="A52" s="4" t="s">
+      <c r="A52" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B52" s="4" t="s">
+      <c r="B52" s="2" t="s">
         <v>114</v>
       </c>
       <c r="C52" s="2" t="s">
@@ -2519,16 +2634,16 @@
       <c r="D52" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E52" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H52" s="3" t="s">
+      <c r="E52" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I52" s="2" t="s">
@@ -2542,10 +2657,10 @@
       <c r="B53" t="s">
         <v>116</v>
       </c>
-      <c r="C53" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D53" s="4" t="s">
+      <c r="C53" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D53" s="2" t="s">
         <v>12</v>
       </c>
       <c r="E53" t="s">
@@ -2557,10 +2672,10 @@
       <c r="G53" t="s">
         <v>11</v>
       </c>
-      <c r="H53" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" s="3" t="s">
+      <c r="H53" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2571,10 +2686,10 @@
       <c r="B54" t="s">
         <v>118</v>
       </c>
-      <c r="C54" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D54" s="4" t="s">
+      <c r="C54" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D54" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E54" t="s">
@@ -2589,7 +2704,7 @@
       <c r="H54" t="s">
         <v>11</v>
       </c>
-      <c r="I54" s="4" t="s">
+      <c r="I54" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2597,7 +2712,7 @@
       <c r="A55" t="s">
         <v>119</v>
       </c>
-      <c r="B55" s="4" t="s">
+      <c r="B55" s="2" t="s">
         <v>120</v>
       </c>
       <c r="C55" t="s">
@@ -2609,7 +2724,7 @@
       <c r="E55" t="s">
         <v>12</v>
       </c>
-      <c r="F55" s="4" t="s">
+      <c r="F55" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G55" t="s">
@@ -2618,7 +2733,7 @@
       <c r="H55" t="s">
         <v>11</v>
       </c>
-      <c r="I55" s="4" t="s">
+      <c r="I55" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2626,13 +2741,13 @@
       <c r="A56" t="s">
         <v>121</v>
       </c>
-      <c r="B56" s="4" t="s">
+      <c r="B56" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C56" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D56" s="4" t="s">
+      <c r="C56" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E56" t="s">
@@ -2647,7 +2762,7 @@
       <c r="H56" t="s">
         <v>12</v>
       </c>
-      <c r="I56" s="4" t="s">
+      <c r="I56" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2655,7 +2770,7 @@
       <c r="A57" t="s">
         <v>123</v>
       </c>
-      <c r="B57" s="4" t="s">
+      <c r="B57" s="2" t="s">
         <v>124</v>
       </c>
       <c r="C57" t="s">
@@ -2713,7 +2828,7 @@
       <c r="A59" t="s">
         <v>127</v>
       </c>
-      <c r="B59" s="4" t="s">
+      <c r="B59" s="2" t="s">
         <v>128</v>
       </c>
       <c r="C59" t="s">
@@ -2734,7 +2849,7 @@
       <c r="H59" t="s">
         <v>11</v>
       </c>
-      <c r="I59" s="3" t="s">
+      <c r="I59" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2760,10 +2875,10 @@
       <c r="G60" t="s">
         <v>11</v>
       </c>
-      <c r="H60" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I60" s="3" t="s">
+      <c r="H60" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2812,7 +2927,7 @@
       <c r="E62" t="s">
         <v>11</v>
       </c>
-      <c r="F62" s="4" t="s">
+      <c r="F62" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G62" t="s">
@@ -2826,16 +2941,16 @@
       </c>
     </row>
     <row r="63" ht="14.25">
-      <c r="A63" s="4" t="s">
+      <c r="A63" s="2" t="s">
         <v>135</v>
       </c>
       <c r="B63" t="s">
         <v>136</v>
       </c>
-      <c r="C63" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D63" s="4" t="s">
+      <c r="C63" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D63" s="2" t="s">
         <v>11</v>
       </c>
       <c r="E63" t="s">
@@ -2867,24 +2982,24 @@
       <c r="D64" t="s">
         <v>12</v>
       </c>
-      <c r="E64" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F64" s="4" t="s">
+      <c r="E64" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F64" s="2" t="s">
         <v>11</v>
       </c>
       <c r="G64" t="s">
         <v>11</v>
       </c>
-      <c r="H64" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" s="3" t="s">
+      <c r="H64" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" s="2" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="65" ht="14.25">
-      <c r="A65" s="4" t="s">
+      <c r="A65" s="2" t="s">
         <v>139</v>
       </c>
       <c r="B65" t="s">
@@ -2896,16 +3011,16 @@
       <c r="D65" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E65" s="3" t="s">
+      <c r="E65" s="2" t="s">
         <v>11</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G65" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H65" s="3" t="s">
+      <c r="G65" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H65" s="2" t="s">
         <v>11</v>
       </c>
       <c r="I65" s="2" t="s">
@@ -2919,25 +3034,25 @@
       <c r="B66" t="s">
         <v>142</v>
       </c>
-      <c r="C66" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E66" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G66" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H66" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I66" s="3" t="s">
+      <c r="C66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -2948,25 +3063,25 @@
       <c r="B67" t="s">
         <v>144</v>
       </c>
-      <c r="C67" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E67" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F67" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="G67" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="H67" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" s="3" t="s">
+      <c r="C67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I67" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -3024,7 +3139,7 @@
       <c r="H69" t="s">
         <v>11</v>
       </c>
-      <c r="I69" s="3" t="s">
+      <c r="I69" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3140,7 +3255,7 @@
       <c r="H73" t="s">
         <v>11</v>
       </c>
-      <c r="I73" s="3" t="s">
+      <c r="I73" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3169,7 +3284,7 @@
       <c r="H74" t="s">
         <v>11</v>
       </c>
-      <c r="I74" s="3" t="s">
+      <c r="I74" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -3227,8 +3342,169 @@
       <c r="H76" t="s">
         <v>11</v>
       </c>
-      <c r="I76" s="3" t="s">
-        <v>11</v>
+      <c r="I76" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="78" s="1" customFormat="1" ht="14.25">
+      <c r="A78" s="1" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="79" ht="14.25">
+      <c r="A79" t="s">
+        <v>166</v>
+      </c>
+      <c r="C79" t="s">
+        <v>167</v>
+      </c>
+      <c r="D79" t="s">
+        <v>168</v>
+      </c>
+      <c r="E79" t="s">
+        <v>169</v>
+      </c>
+      <c r="F79" t="s">
+        <v>167</v>
+      </c>
+      <c r="G79" t="s">
+        <v>169</v>
+      </c>
+      <c r="H79" t="s">
+        <v>168</v>
+      </c>
+      <c r="I79" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="80" ht="14.25">
+      <c r="A80" t="s">
+        <v>170</v>
+      </c>
+      <c r="C80" t="s">
+        <v>171</v>
+      </c>
+      <c r="D80" t="s">
+        <v>172</v>
+      </c>
+      <c r="E80" t="s">
+        <v>172</v>
+      </c>
+      <c r="F80" t="s">
+        <v>173</v>
+      </c>
+      <c r="G80" t="s">
+        <v>174</v>
+      </c>
+      <c r="H80" t="s">
+        <v>174</v>
+      </c>
+      <c r="I80" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="81" ht="14.25">
+      <c r="A81" t="s">
+        <v>176</v>
+      </c>
+      <c r="C81" t="s">
+        <v>177</v>
+      </c>
+      <c r="D81" t="s">
+        <v>178</v>
+      </c>
+      <c r="E81" t="s">
+        <v>179</v>
+      </c>
+      <c r="F81" t="s">
+        <v>180</v>
+      </c>
+      <c r="G81" t="s">
+        <v>181</v>
+      </c>
+      <c r="H81" t="s">
+        <v>182</v>
+      </c>
+      <c r="I81" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="82" ht="14.25">
+      <c r="A82" t="s">
+        <v>184</v>
+      </c>
+      <c r="C82" t="s">
+        <v>185</v>
+      </c>
+      <c r="D82" t="s">
+        <v>186</v>
+      </c>
+      <c r="E82" t="s">
+        <v>187</v>
+      </c>
+      <c r="F82" t="s">
+        <v>188</v>
+      </c>
+      <c r="G82" t="s">
+        <v>189</v>
+      </c>
+      <c r="H82" t="s">
+        <v>190</v>
+      </c>
+      <c r="I82" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="83" ht="14.25">
+      <c r="A83" t="s">
+        <v>192</v>
+      </c>
+      <c r="C83" t="s">
+        <v>193</v>
+      </c>
+      <c r="D83" t="s">
+        <v>194</v>
+      </c>
+      <c r="E83" t="s">
+        <v>195</v>
+      </c>
+      <c r="F83" t="s">
+        <v>186</v>
+      </c>
+      <c r="G83" t="s">
+        <v>195</v>
+      </c>
+      <c r="H83" t="s">
+        <v>194</v>
+      </c>
+      <c r="I83" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="84" ht="14.25">
+      <c r="A84" t="s">
+        <v>196</v>
+      </c>
+      <c r="C84" t="s">
+        <v>197</v>
+      </c>
+      <c r="D84" t="s">
+        <v>198</v>
+      </c>
+      <c r="E84" t="s">
+        <v>199</v>
+      </c>
+      <c r="F84" t="s">
+        <v>200</v>
+      </c>
+      <c r="G84" t="s">
+        <v>201</v>
+      </c>
+      <c r="H84" t="s">
+        <v>202</v>
+      </c>
+      <c r="I84" t="s">
+        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3243,7 +3519,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{00E300EB-008A-4AE4-BB37-00430039004C}">
+          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{008F00BC-00CA-44A9-A888-00DB0089008C}">
             <xm:f>LEFT(C1,LEN("yes"))="yes"</xm:f>
             <x14:dxf>
               <font>
@@ -3260,7 +3536,7 @@
           <xm:sqref>C2:I76</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="1" text="no" id="{00AF00E1-004A-4792-80BE-002500F70039}">
+          <x14:cfRule type="beginsWith" priority="1" text="no" id="{00B80052-008C-4D2D-A662-006B005800FB}">
             <xm:f>LEFT(C2,LEN("no"))="no"</xm:f>
             <x14:dxf>
               <font>

</xml_diff>

<commit_message>
chore: update feature comparison table
</commit_message>
<xml_diff>
--- a/Feature_Comparison.xlsx
+++ b/Feature_Comparison.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="210">
   <si>
     <t>Feature</t>
   </si>
@@ -315,30 +315,36 @@
     <t xml:space="preserve">which disconnected skeleton component each segment belongs to</t>
   </si>
   <si>
-    <t>per_segment_diameter</t>
+    <t>per_segment_endpoint_image_coords</t>
+  </si>
+  <si>
+    <t xml:space="preserve">image-space coords of each segments source and dest. endpoints</t>
+  </si>
+  <si>
+    <t>per_segment_euclidean_distance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">straight-line end-to-end distance for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_is_main_branch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">whether segment belongs to the longest shortest path within its skeleton component</t>
+  </si>
+  <si>
+    <t>per_segment_max_diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">max vessel diameter measured along centerlines for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_mean_diameter</t>
   </si>
   <si>
     <t xml:space="preserve">mean vessel diameter measured along centerlines for each segment</t>
   </si>
   <si>
-    <t>per_segment_endpoint_image_coords</t>
-  </si>
-  <si>
-    <t xml:space="preserve">image-space coords of each segments source and dest. endpoints</t>
-  </si>
-  <si>
-    <t>per_segment_euclidean_distance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">straight-line end-to-end distance for each segment</t>
-  </si>
-  <si>
-    <t>per_segment_is_main_branch</t>
-  </si>
-  <si>
-    <t xml:space="preserve">whether segment belongs to the longest shortest path within its skeleton component</t>
-  </si>
-  <si>
     <t>per_segment_mean_pixel_intensity</t>
   </si>
   <si>
@@ -351,19 +357,31 @@
     <t xml:space="preserve">average radius along the segment centerline for each segment</t>
   </si>
   <si>
+    <t>per_segment_min_diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">min vessel diameter measured along centerlines for each segment</t>
+  </si>
+  <si>
     <t>per_segment_min_radius</t>
   </si>
   <si>
     <t xml:space="preserve">minimum radius along the segment for each segment</t>
   </si>
   <si>
-    <t>per_segment_pixel_intensity_stddev</t>
+    <t>per_segment_pixel_intensity_std</t>
   </si>
   <si>
     <t xml:space="preserve">standard deviation of image intensity along each segment</t>
   </si>
   <si>
-    <t>per_segment_radius_stddev</t>
+    <t>per_segment_std_diameter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">std dev of vessel diameter measured along centerlines for each segment</t>
+  </si>
+  <si>
+    <t>per_segment_std_radius</t>
   </si>
   <si>
     <t xml:space="preserve">standard deviation of radii along the segment for each segment</t>
@@ -486,13 +504,13 @@
     <t>vessel_area</t>
   </si>
   <si>
-    <t xml:space="preserve">pixels/um^2 classified as vessel</t>
+    <t xml:space="preserve">pixels/voxels classified as vessel</t>
   </si>
   <si>
     <t>vessel_area_fraction</t>
   </si>
   <si>
-    <t xml:space="preserve">fraction of image pixels classified as vessel</t>
+    <t xml:space="preserve">fraction of image pixels/voxels classified as vessel</t>
   </si>
   <si>
     <t xml:space="preserve">yes (Total network volume (3D) or total PAF (2D) is reported as “Volume” / “Percent Area Fraction (PAF) %)</t>
@@ -669,12 +687,21 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="8">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1135,7 +1162,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr baseColWidth="9" defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="27.7109375"/>
+    <col customWidth="1" min="1" max="1" width="38.57421875"/>
     <col customWidth="1" min="2" max="2" width="51.421875"/>
     <col customWidth="1" min="4" max="4" width="12.421875"/>
     <col customWidth="1" min="5" max="5" width="13.28125"/>
@@ -1486,7 +1513,7 @@
         <v>12</v>
       </c>
       <c r="I12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="13" ht="14.25">
@@ -1573,7 +1600,7 @@
         <v>12</v>
       </c>
       <c r="I15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" ht="14.25">
@@ -1631,7 +1658,7 @@
         <v>11</v>
       </c>
       <c r="I17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" ht="14.25">
@@ -1805,7 +1832,7 @@
         <v>11</v>
       </c>
       <c r="I23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="14.25">
@@ -1892,7 +1919,7 @@
         <v>11</v>
       </c>
       <c r="I26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27" ht="14.25">
@@ -2431,7 +2458,7 @@
         <v>11</v>
       </c>
       <c r="E45" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F45" t="s">
         <v>11</v>
@@ -2440,10 +2467,10 @@
         <v>11</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I45" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="46" ht="14.25">
@@ -2472,7 +2499,7 @@
         <v>12</v>
       </c>
       <c r="I46" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="47" ht="14.25">
@@ -2501,40 +2528,40 @@
         <v>12</v>
       </c>
       <c r="I47" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48" ht="14.25">
-      <c r="A48" t="s">
+      <c r="A48" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="C48" t="s">
-        <v>11</v>
-      </c>
-      <c r="D48" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" t="s">
-        <v>11</v>
-      </c>
-      <c r="F48" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" t="s">
-        <v>11</v>
-      </c>
-      <c r="H48" t="s">
-        <v>12</v>
-      </c>
-      <c r="I48" t="s">
-        <v>11</v>
+      <c r="C48" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I48" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="49" ht="14.25">
-      <c r="A49" t="s">
+      <c r="A49" s="5" t="s">
         <v>107</v>
       </c>
       <c r="B49" t="s">
@@ -2547,7 +2574,7 @@
         <v>11</v>
       </c>
       <c r="E49" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F49" t="s">
         <v>11</v>
@@ -2556,10 +2583,10 @@
         <v>11</v>
       </c>
       <c r="H49" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I49" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="50" ht="14.25">
@@ -2573,7 +2600,7 @@
         <v>11</v>
       </c>
       <c r="D50" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E50" t="s">
         <v>11</v>
@@ -2585,10 +2612,10 @@
         <v>11</v>
       </c>
       <c r="H50" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I50" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="51" ht="14.25">
@@ -2617,36 +2644,36 @@
         <v>11</v>
       </c>
       <c r="I51" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="52" ht="14.25">
-      <c r="A52" t="s">
+      <c r="A52" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B52" t="s">
+      <c r="B52" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C52" t="s">
-        <v>11</v>
-      </c>
-      <c r="D52" t="s">
-        <v>11</v>
-      </c>
-      <c r="E52" t="s">
-        <v>11</v>
-      </c>
-      <c r="F52" t="s">
-        <v>11</v>
-      </c>
-      <c r="G52" t="s">
-        <v>11</v>
-      </c>
-      <c r="H52" t="s">
-        <v>12</v>
-      </c>
-      <c r="I52" t="s">
-        <v>11</v>
+      <c r="C52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I52" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="53" ht="14.25">
@@ -2675,7 +2702,7 @@
         <v>11</v>
       </c>
       <c r="I53" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="54" ht="14.25">
@@ -2692,7 +2719,7 @@
         <v>11</v>
       </c>
       <c r="E54" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F54" t="s">
         <v>11</v>
@@ -2704,40 +2731,40 @@
         <v>12</v>
       </c>
       <c r="I54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="55" ht="14.25">
-      <c r="A55" t="s">
+      <c r="A55" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="B55" t="s">
+      <c r="B55" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="C55" t="s">
-        <v>11</v>
-      </c>
-      <c r="D55" t="s">
-        <v>11</v>
-      </c>
-      <c r="E55" t="s">
-        <v>12</v>
-      </c>
-      <c r="F55" t="s">
-        <v>11</v>
-      </c>
-      <c r="G55" t="s">
-        <v>11</v>
-      </c>
-      <c r="H55" t="s">
-        <v>12</v>
-      </c>
-      <c r="I55" t="s">
-        <v>11</v>
+      <c r="C55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" s="5" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="56" ht="14.25">
-      <c r="A56" t="s">
+      <c r="A56" s="5" t="s">
         <v>121</v>
       </c>
       <c r="B56" t="s">
@@ -2747,7 +2774,7 @@
         <v>11</v>
       </c>
       <c r="D56" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E56" t="s">
         <v>11</v>
@@ -2759,7 +2786,7 @@
         <v>11</v>
       </c>
       <c r="H56" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I56" t="s">
         <v>12</v>
@@ -2776,7 +2803,7 @@
         <v>11</v>
       </c>
       <c r="D57" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E57" t="s">
         <v>12</v>
@@ -2805,7 +2832,7 @@
         <v>11</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E58" t="s">
         <v>12</v>
@@ -2817,7 +2844,7 @@
         <v>11</v>
       </c>
       <c r="H58" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I58" t="s">
         <v>11</v>
@@ -2834,7 +2861,7 @@
         <v>11</v>
       </c>
       <c r="D59" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E59" t="s">
         <v>11</v>
@@ -2846,10 +2873,10 @@
         <v>11</v>
       </c>
       <c r="H59" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I59" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="60" ht="14.25">
@@ -2866,7 +2893,7 @@
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F60" t="s">
         <v>11</v>
@@ -2875,10 +2902,10 @@
         <v>11</v>
       </c>
       <c r="H60" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I60" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="61" ht="14.25">
@@ -2889,7 +2916,7 @@
         <v>132</v>
       </c>
       <c r="C61" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
@@ -2904,10 +2931,10 @@
         <v>11</v>
       </c>
       <c r="H61" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I61" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" ht="14.25">
@@ -2936,7 +2963,7 @@
         <v>11</v>
       </c>
       <c r="I62" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="63" ht="14.25">
@@ -2950,13 +2977,13 @@
         <v>11</v>
       </c>
       <c r="D63" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E63" t="s">
         <v>11</v>
       </c>
       <c r="F63" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G63" t="s">
         <v>11</v>
@@ -2976,13 +3003,13 @@
         <v>138</v>
       </c>
       <c r="C64" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D64" t="s">
         <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F64" t="s">
         <v>11</v>
@@ -2991,10 +3018,10 @@
         <v>11</v>
       </c>
       <c r="H64" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I64" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="65" ht="14.25">
@@ -3008,7 +3035,7 @@
         <v>11</v>
       </c>
       <c r="D65" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
@@ -3020,7 +3047,7 @@
         <v>11</v>
       </c>
       <c r="H65" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I65" t="s">
         <v>11</v>
@@ -3043,13 +3070,13 @@
         <v>11</v>
       </c>
       <c r="F66" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G66" t="s">
         <v>11</v>
       </c>
       <c r="H66" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I66" t="s">
         <v>11</v>
@@ -3066,7 +3093,7 @@
         <v>11</v>
       </c>
       <c r="D67" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E67" t="s">
         <v>11</v>
@@ -3078,7 +3105,7 @@
         <v>11</v>
       </c>
       <c r="H67" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I67" t="s">
         <v>11</v>
@@ -3095,10 +3122,10 @@
         <v>11</v>
       </c>
       <c r="D68" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E68" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F68" t="s">
         <v>11</v>
@@ -3124,7 +3151,7 @@
         <v>11</v>
       </c>
       <c r="D69" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E69" t="s">
         <v>11</v>
@@ -3136,7 +3163,7 @@
         <v>11</v>
       </c>
       <c r="H69" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I69" t="s">
         <v>11</v>
@@ -3159,7 +3186,7 @@
         <v>11</v>
       </c>
       <c r="F70" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G70" t="s">
         <v>11</v>
@@ -3182,10 +3209,10 @@
         <v>11</v>
       </c>
       <c r="D71" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E71" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F71" t="s">
         <v>11</v>
@@ -3197,7 +3224,7 @@
         <v>12</v>
       </c>
       <c r="I71" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="72" ht="14.25">
@@ -3211,7 +3238,7 @@
         <v>11</v>
       </c>
       <c r="D72" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E72" t="s">
         <v>11</v>
@@ -3223,10 +3250,10 @@
         <v>11</v>
       </c>
       <c r="H72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I72" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="73" ht="14.25">
@@ -3252,7 +3279,7 @@
         <v>11</v>
       </c>
       <c r="H73" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I73" t="s">
         <v>11</v>
@@ -3266,10 +3293,10 @@
         <v>158</v>
       </c>
       <c r="C74" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D74" t="s">
-        <v>159</v>
+        <v>11</v>
       </c>
       <c r="E74" t="s">
         <v>11</v>
@@ -3281,30 +3308,30 @@
         <v>11</v>
       </c>
       <c r="H74" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I74" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="75" ht="14.25">
       <c r="A75" t="s">
+        <v>159</v>
+      </c>
+      <c r="B75" t="s">
         <v>160</v>
       </c>
-      <c r="B75" t="s">
-        <v>161</v>
-      </c>
       <c r="C75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D75" t="s">
-        <v>162</v>
+        <v>11</v>
       </c>
       <c r="E75" t="s">
         <v>11</v>
       </c>
       <c r="F75" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G75" t="s">
         <v>11</v>
@@ -3318,197 +3345,284 @@
     </row>
     <row r="76" ht="14.25">
       <c r="A76" t="s">
+        <v>161</v>
+      </c>
+      <c r="B76" t="s">
+        <v>162</v>
+      </c>
+      <c r="C76" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" t="s">
+        <v>11</v>
+      </c>
+      <c r="E76" t="s">
+        <v>11</v>
+      </c>
+      <c r="F76" t="s">
+        <v>12</v>
+      </c>
+      <c r="G76" t="s">
+        <v>11</v>
+      </c>
+      <c r="H76" t="s">
+        <v>11</v>
+      </c>
+      <c r="I76" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="77" ht="14.25">
+      <c r="A77" t="s">
         <v>163</v>
       </c>
-      <c r="B76" t="s">
+      <c r="B77" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="C76" t="s">
-        <v>12</v>
-      </c>
-      <c r="D76" t="s">
-        <v>11</v>
-      </c>
-      <c r="E76" t="s">
-        <v>11</v>
-      </c>
-      <c r="F76" t="s">
-        <v>11</v>
-      </c>
-      <c r="G76" t="s">
-        <v>11</v>
-      </c>
-      <c r="H76" t="s">
-        <v>11</v>
-      </c>
-      <c r="I76" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="78" s="1" customFormat="1" ht="14.25">
-      <c r="A78" s="1" t="s">
+      <c r="C77" t="s">
+        <v>12</v>
+      </c>
+      <c r="D77" t="s">
         <v>165</v>
+      </c>
+      <c r="E77" t="s">
+        <v>11</v>
+      </c>
+      <c r="F77" t="s">
+        <v>11</v>
+      </c>
+      <c r="G77" t="s">
+        <v>11</v>
+      </c>
+      <c r="H77" t="s">
+        <v>11</v>
+      </c>
+      <c r="I77" s="7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="78" s="0" customFormat="1" ht="14.25">
+      <c r="A78" t="s">
+        <v>166</v>
+      </c>
+      <c r="B78" t="s">
+        <v>167</v>
+      </c>
+      <c r="C78" t="s">
+        <v>12</v>
+      </c>
+      <c r="D78" t="s">
+        <v>168</v>
+      </c>
+      <c r="E78" t="s">
+        <v>11</v>
+      </c>
+      <c r="F78" t="s">
+        <v>12</v>
+      </c>
+      <c r="G78" t="s">
+        <v>11</v>
+      </c>
+      <c r="H78" t="s">
+        <v>12</v>
+      </c>
+      <c r="I78" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="79" ht="14.25">
       <c r="A79" t="s">
-        <v>166</v>
+        <v>169</v>
+      </c>
+      <c r="B79" t="s">
+        <v>170</v>
       </c>
       <c r="C79" t="s">
-        <v>167</v>
+        <v>12</v>
       </c>
       <c r="D79" t="s">
-        <v>168</v>
+        <v>11</v>
       </c>
       <c r="E79" t="s">
-        <v>169</v>
+        <v>11</v>
       </c>
       <c r="F79" t="s">
-        <v>167</v>
+        <v>11</v>
       </c>
       <c r="G79" t="s">
-        <v>169</v>
+        <v>11</v>
       </c>
       <c r="H79" t="s">
-        <v>168</v>
+        <v>11</v>
       </c>
       <c r="I79" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="80" ht="14.25">
-      <c r="A80" t="s">
-        <v>170</v>
-      </c>
-      <c r="C80" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="82" ht="14.25">
+      <c r="A82" s="1" t="s">
         <v>171</v>
-      </c>
-      <c r="D80" t="s">
-        <v>172</v>
-      </c>
-      <c r="E80" t="s">
-        <v>173</v>
-      </c>
-      <c r="F80" t="s">
-        <v>174</v>
-      </c>
-      <c r="G80" t="s">
-        <v>175</v>
-      </c>
-      <c r="H80" t="s">
-        <v>176</v>
-      </c>
-      <c r="I80" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="81" ht="14.25">
-      <c r="A81" t="s">
-        <v>178</v>
-      </c>
-      <c r="C81" t="s">
-        <v>179</v>
-      </c>
-      <c r="D81" t="s">
-        <v>180</v>
-      </c>
-      <c r="E81" t="s">
-        <v>181</v>
-      </c>
-      <c r="F81" t="s">
-        <v>182</v>
-      </c>
-      <c r="G81" t="s">
-        <v>183</v>
-      </c>
-      <c r="H81" t="s">
-        <v>184</v>
-      </c>
-      <c r="I81" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="82" ht="14.25">
-      <c r="A82" t="s">
-        <v>186</v>
-      </c>
-      <c r="C82" t="s">
-        <v>187</v>
-      </c>
-      <c r="D82" t="s">
-        <v>188</v>
-      </c>
-      <c r="E82" t="s">
-        <v>188</v>
-      </c>
-      <c r="F82" t="s">
-        <v>189</v>
-      </c>
-      <c r="G82" t="s">
-        <v>190</v>
-      </c>
-      <c r="H82" t="s">
-        <v>191</v>
-      </c>
-      <c r="I82" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="83" ht="14.25">
       <c r="A83" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="C83" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="D83" t="s">
-        <v>194</v>
+        <v>174</v>
       </c>
       <c r="E83" t="s">
-        <v>195</v>
+        <v>175</v>
       </c>
       <c r="F83" t="s">
-        <v>196</v>
+        <v>173</v>
       </c>
       <c r="G83" t="s">
-        <v>197</v>
+        <v>175</v>
       </c>
       <c r="H83" t="s">
-        <v>198</v>
+        <v>174</v>
       </c>
       <c r="I83" t="s">
-        <v>199</v>
+        <v>174</v>
       </c>
     </row>
     <row r="84" ht="14.25">
       <c r="A84" t="s">
+        <v>176</v>
+      </c>
+      <c r="C84" t="s">
+        <v>177</v>
+      </c>
+      <c r="D84" t="s">
+        <v>178</v>
+      </c>
+      <c r="E84" t="s">
+        <v>179</v>
+      </c>
+      <c r="F84" t="s">
+        <v>180</v>
+      </c>
+      <c r="G84" t="s">
+        <v>181</v>
+      </c>
+      <c r="H84" t="s">
+        <v>182</v>
+      </c>
+      <c r="I84" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="85" ht="14.25">
+      <c r="A85" t="s">
+        <v>184</v>
+      </c>
+      <c r="C85" t="s">
+        <v>185</v>
+      </c>
+      <c r="D85" t="s">
+        <v>186</v>
+      </c>
+      <c r="E85" t="s">
+        <v>187</v>
+      </c>
+      <c r="F85" t="s">
+        <v>188</v>
+      </c>
+      <c r="G85" t="s">
+        <v>189</v>
+      </c>
+      <c r="H85" t="s">
+        <v>190</v>
+      </c>
+      <c r="I85" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="86" ht="14.25">
+      <c r="A86" t="s">
+        <v>192</v>
+      </c>
+      <c r="C86" t="s">
+        <v>193</v>
+      </c>
+      <c r="D86" t="s">
+        <v>194</v>
+      </c>
+      <c r="E86" t="s">
+        <v>194</v>
+      </c>
+      <c r="F86" t="s">
+        <v>195</v>
+      </c>
+      <c r="G86" t="s">
+        <v>196</v>
+      </c>
+      <c r="H86" t="s">
+        <v>197</v>
+      </c>
+      <c r="I86" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="87" ht="14.25">
+      <c r="A87" t="s">
+        <v>198</v>
+      </c>
+      <c r="C87" t="s">
+        <v>199</v>
+      </c>
+      <c r="D87" t="s">
         <v>200</v>
       </c>
-      <c r="C84" t="s">
+      <c r="E87" t="s">
         <v>201</v>
       </c>
-      <c r="D84" t="s">
+      <c r="F87" t="s">
         <v>202</v>
       </c>
-      <c r="E84" t="s">
+      <c r="G87" t="s">
         <v>203</v>
       </c>
-      <c r="F84" t="s">
-        <v>194</v>
-      </c>
-      <c r="G84" t="s">
-        <v>203</v>
-      </c>
-      <c r="H84" t="s">
-        <v>194</v>
-      </c>
-      <c r="I84" t="s">
-        <v>202</v>
+      <c r="H87" t="s">
+        <v>204</v>
+      </c>
+      <c r="I87" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="88" ht="14.25">
+      <c r="A88" t="s">
+        <v>206</v>
+      </c>
+      <c r="C88" t="s">
+        <v>207</v>
+      </c>
+      <c r="D88" t="s">
+        <v>208</v>
+      </c>
+      <c r="E88" t="s">
+        <v>209</v>
+      </c>
+      <c r="F88" t="s">
+        <v>200</v>
+      </c>
+      <c r="G88" t="s">
+        <v>209</v>
+      </c>
+      <c r="H88" t="s">
+        <v>200</v>
+      </c>
+      <c r="I88" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
-  <sortState ref="A79:I84" columnSort="0">
-    <sortCondition sortBy="value" descending="0" ref="A79:A84"/>
+  <sortState ref="A2:I79" columnSort="0">
+    <sortCondition sortBy="value" descending="0" ref="A2:A79"/>
   </sortState>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -3518,7 +3632,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{00C90012-0095-44BD-B88F-002F0030001A}">
+          <x14:cfRule type="beginsWith" priority="2" text="yes" id="{005F0041-00D7-4A9D-9CAD-008000C90087}">
             <xm:f>LEFT(C1,LEN("yes"))="yes"</xm:f>
             <x14:dxf>
               <font>
@@ -3532,10 +3646,10 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>C2:G76 H2:H76 I2:I76</xm:sqref>
+          <xm:sqref>C2:I79</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="1" text="no" id="{0095006D-00E8-42A2-B743-002500EF0079}">
+          <x14:cfRule type="beginsWith" priority="1" text="no" id="{00E000E8-009F-41BD-BA9D-000800BD00F3}">
             <xm:f>LEFT(C2,LEN("no"))="no"</xm:f>
             <x14:dxf>
               <font>
@@ -3549,7 +3663,7 @@
               </fill>
             </x14:dxf>
           </x14:cfRule>
-          <xm:sqref>C2:G76 H2:H76 I2:I76</xm:sqref>
+          <xm:sqref>C2:I79</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
chore: update feature table
</commit_message>
<xml_diff>
--- a/Feature_Comparison.xlsx
+++ b/Feature_Comparison.xlsx
@@ -1540,7 +1540,7 @@
         <v>11</v>
       </c>
       <c r="I13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="14" ht="14.25">
@@ -1569,7 +1569,7 @@
         <v>11</v>
       </c>
       <c r="I14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" ht="14.25">
@@ -1627,7 +1627,7 @@
         <v>12</v>
       </c>
       <c r="I16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" ht="14.25">
@@ -1946,7 +1946,7 @@
         <v>11</v>
       </c>
       <c r="I27" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="28" ht="14.25">
@@ -1975,7 +1975,7 @@
         <v>11</v>
       </c>
       <c r="I28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="29" ht="14.25">
@@ -2149,7 +2149,7 @@
         <v>12</v>
       </c>
       <c r="I34" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" ht="14.25">
@@ -2526,7 +2526,7 @@
         <v>12</v>
       </c>
       <c r="I47" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="48" ht="14.25">
@@ -2845,7 +2845,7 @@
         <v>12</v>
       </c>
       <c r="I58" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="59" ht="14.25">
@@ -3630,7 +3630,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="3" text="yes" id="{009A00AA-00B0-42DB-97DD-0087001600FF}">
+          <x14:cfRule type="beginsWith" priority="3" text="yes" id="{00800093-008A-4C21-9A56-005A000300AD}">
             <xm:f>LEFT(C1,LEN("yes"))="yes"</xm:f>
             <x14:dxf>
               <font>
@@ -3647,7 +3647,7 @@
           <xm:sqref>C2:I79</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="2" text="no" id="{00DD00B9-00CA-4E57-8D27-005800360018}">
+          <x14:cfRule type="beginsWith" priority="2" text="no" id="{008A00F3-0016-4415-A3D6-0064006400D6}">
             <xm:f>LEFT(C2,LEN("no"))="no"</xm:f>
             <x14:dxf>
               <font>
@@ -3664,7 +3664,7 @@
           <xm:sqref>C2:I79</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="1" text="nope" id="{00FA000A-0090-4179-BF32-00F6007100FC}">
+          <x14:cfRule type="beginsWith" priority="1" text="nope" id="{00E0004B-00D8-4952-AF5F-0028006900A5}">
             <xm:f>LEFT(I1,LEN("nope"))="nope"</xm:f>
             <x14:dxf>
               <font>

</xml_diff>

<commit_message>
docs: add part about graph construction and features
</commit_message>
<xml_diff>
--- a/Feature_Comparison.xlsx
+++ b/Feature_Comparison.xlsx
@@ -48,7 +48,7 @@
     <t>alignment_coherency_percent</t>
   </si>
   <si>
-    <t xml:space="preserve">global fibre alignment coherency (0–100%)</t>
+    <t xml:space="preserve">global fibre alignment coherency (0-100%)</t>
   </si>
   <si>
     <t>no</t>
@@ -57,7 +57,7 @@
     <t>yes</t>
   </si>
   <si>
-    <t>nope</t>
+    <t>omitted</t>
   </si>
   <si>
     <t>branchpoint_count</t>
@@ -2294,7 +2294,7 @@
         <v>12</v>
       </c>
       <c r="I39" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="40" ht="14.25">
@@ -2323,7 +2323,7 @@
         <v>12</v>
       </c>
       <c r="I40" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="41" ht="14.25">
@@ -2410,7 +2410,7 @@
         <v>12</v>
       </c>
       <c r="I43" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="44" ht="14.25">
@@ -2439,7 +2439,7 @@
         <v>12</v>
       </c>
       <c r="I44" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="45" ht="14.25">
@@ -3630,7 +3630,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="3" text="yes" id="{00800093-008A-4C21-9A56-005A000300AD}">
+          <x14:cfRule type="beginsWith" priority="3" text="yes" id="{008C0064-0071-4029-845C-00A5006B0084}">
             <xm:f>LEFT(C1,LEN("yes"))="yes"</xm:f>
             <x14:dxf>
               <font>
@@ -3647,7 +3647,7 @@
           <xm:sqref>C2:I79</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="2" text="no" id="{008A00F3-0016-4415-A3D6-0064006400D6}">
+          <x14:cfRule type="beginsWith" priority="2" text="no" id="{00E20074-00F7-450F-A3D4-00A7009A00D3}">
             <xm:f>LEFT(C2,LEN("no"))="no"</xm:f>
             <x14:dxf>
               <font>
@@ -3664,8 +3664,8 @@
           <xm:sqref>C2:I79</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="beginsWith" priority="1" text="nope" id="{00E0004B-00D8-4952-AF5F-0028006900A5}">
-            <xm:f>LEFT(I1,LEN("nope"))="nope"</xm:f>
+          <x14:cfRule type="beginsWith" priority="1" text="omitted" id="{00C400BD-00D1-4E28-8B1C-004E00550056}">
+            <xm:f>LEFT(I1,LEN("omitted"))="omitted"</xm:f>
             <x14:dxf>
               <font>
                 <color rgb="FF9C5700"/>

</xml_diff>